<commit_message>
Data analysis: data (updated)
</commit_message>
<xml_diff>
--- a/data_analysis/data.xlsx
+++ b/data_analysis/data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t xml:space="preserve">waktu</t>
   </si>
@@ -46,6 +46,9 @@
     <t xml:space="preserve">2026-06-08 09:05:08</t>
   </si>
   <si>
+    <t xml:space="preserve">Rp 6000</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-06-08 10:30:20</t>
   </si>
   <si>
@@ -58,7 +61,7 @@
     <t xml:space="preserve">Sinkong Keju</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-06-08 12:04:29</t>
+    <t xml:space="preserve">08/06/2026 12:04</t>
   </si>
   <si>
     <t xml:space="preserve">2026-06-08 12:08:20</t>
@@ -347,19 +350,16 @@
       <c r="C4" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="D4" s="0" t="n">
-        <v>6000</v>
+      <c r="D4" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="0" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D5" s="0" t="n">
         <v>5000</v>
@@ -367,10 +367,10 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="0" t="n">
         <v>1</v>
@@ -381,7 +381,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>6</v>
@@ -395,10 +395,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" s="0" t="n">
         <v>1</v>
@@ -409,10 +409,10 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" s="0" t="n">
         <v>4</v>
@@ -423,10 +423,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" s="0" t="n">
         <v>5</v>
@@ -437,7 +437,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Data analysis: data (updated), load, clean, clean data
</commit_message>
<xml_diff>
--- a/data_analysis/data.xlsx
+++ b/data_analysis/data.xlsx
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Sinkong Keju</t>
   </si>
   <si>
-    <t xml:space="preserve">08/06/2026 12:04</t>
+    <t xml:space="preserve">08/06/2026 12:04:29</t>
   </si>
   <si>
     <t xml:space="preserve">2026-06-08 12:08:20</t>
@@ -445,9 +445,6 @@
       <c r="C11" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="0" t="n">
-        <v>6000</v>
-      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>